<commit_message>
rxns up to cam_ca4 binding to camkii and phospho
</commit_message>
<xml_diff>
--- a/rxns_table.xlsx
+++ b/rxns_table.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="27830"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="27928"/>
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\PhD_2023\CaMKII_hexa_bgnl_to_mcell\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{2A618A38-8E02-40BE-856D-6A386AE4F1E7}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{85619136-64D9-4EE1-9C53-2A04689AEF0B}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-57720" yWindow="-120" windowWidth="29040" windowHeight="15840" xr2:uid="{4B4FB280-5B08-406D-B059-D87F72317E26}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15840" xr2:uid="{4B4FB280-5B08-406D-B059-D87F72317E26}"/>
   </bookViews>
   <sheets>
     <sheet name="rxns_table" sheetId="1" r:id="rId1"/>
@@ -38,6 +38,7 @@
     <author>tc={67578144-E3EC-4152-8729-1B44EEC1002D}</author>
     <author>tc={6F7C1780-1EE0-4B0C-B03B-9322192D7EC2}</author>
     <author>tc={802EEB37-19A7-4071-9209-8ED3C607D4E8}</author>
+    <author>tc={CDBBDAF0-DC8A-4716-92BA-AC44BC912388}</author>
     <author>tc={B6F8C469-337C-40BE-B2DC-A13B6B68197A}</author>
     <author>Susana Roman</author>
     <author>tc={6C2818CD-9DCB-407F-A713-A0F009955982}</author>
@@ -72,7 +73,15 @@
 </t>
       </text>
     </comment>
-    <comment ref="B18" authorId="3" shapeId="0" xr:uid="{B6F8C469-337C-40BE-B2DC-A13B6B68197A}">
+    <comment ref="E15" authorId="3" shapeId="0" xr:uid="{CDBBDAF0-DC8A-4716-92BA-AC44BC912388}">
+      <text>
+        <t>[Threaded comment]
+Your version of Excel allows you to read this threaded comment; however, any edits to it will get removed if the file is opened in a newer version of Excel. Learn more: https://go.microsoft.com/fwlink/?linkid=870924
+Comment:
+    Divide it by 2e10-3</t>
+      </text>
+    </comment>
+    <comment ref="B18" authorId="4" shapeId="0" xr:uid="{B6F8C469-337C-40BE-B2DC-A13B6B68197A}">
       <text>
         <t>[Threaded comment]
 Your version of Excel allows you to read this threaded comment; however, any edits to it will get removed if the file is opened in a newer version of Excel. Learn more: https://go.microsoft.com/fwlink/?linkid=870924
@@ -80,7 +89,7 @@
     Not modelled currently; we specify different off rates depending on whether camkii is P or not.</t>
       </text>
     </comment>
-    <comment ref="P19" authorId="4" shapeId="0" xr:uid="{7C16AAE1-EC76-4DE7-BC28-A2AA54E7931D}">
+    <comment ref="P19" authorId="5" shapeId="0" xr:uid="{7C16AAE1-EC76-4DE7-BC28-A2AA54E7931D}">
       <text>
         <r>
           <rPr>
@@ -104,7 +113,7 @@
         </r>
       </text>
     </comment>
-    <comment ref="N22" authorId="4" shapeId="0" xr:uid="{D783E934-AE8E-45F6-BF32-CFA5F3DEAB20}">
+    <comment ref="N22" authorId="5" shapeId="0" xr:uid="{D783E934-AE8E-45F6-BF32-CFA5F3DEAB20}">
       <text>
         <r>
           <rPr>
@@ -128,7 +137,7 @@
         </r>
       </text>
     </comment>
-    <comment ref="P25" authorId="5" shapeId="0" xr:uid="{6C2818CD-9DCB-407F-A713-A0F009955982}">
+    <comment ref="P25" authorId="6" shapeId="0" xr:uid="{6C2818CD-9DCB-407F-A713-A0F009955982}">
       <text>
         <t>[Threaded comment]
 Your version of Excel allows you to read this threaded comment; however, any edits to it will get removed if the file is opened in a newer version of Excel. Learn more: https://go.microsoft.com/fwlink/?linkid=870924
@@ -155,12 +164,6 @@
     <t>CaMKII subunits active/inactive flicker</t>
   </si>
   <si>
-    <t>kon_CaMKII_act</t>
-  </si>
-  <si>
-    <t>koff_CaMKII_inact</t>
-  </si>
-  <si>
     <t>kon_CaM_Ca4_CaMKII</t>
   </si>
   <si>
@@ -312,13 +315,19 @@
   </si>
   <si>
     <t>Rellos et al., 2010</t>
+  </si>
+  <si>
+    <t>kon_CaMKII_open</t>
+  </si>
+  <si>
+    <t>koff_CaMKII_close</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="26" x14ac:knownFonts="1">
+  <fonts count="27" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -505,6 +514,12 @@
       <color indexed="81"/>
       <name val="Tahoma"/>
       <family val="2"/>
+    </font>
+    <font>
+      <sz val="9"/>
+      <color indexed="81"/>
+      <name val="Tahoma"/>
+      <charset val="1"/>
     </font>
   </fonts>
   <fills count="41">
@@ -1364,6 +1379,9 @@
     <text xml:space="preserve">Range 1.6 and 3.4×106 Mol−1
 </text>
   </threadedComment>
+  <threadedComment ref="E15" dT="2024-09-13T10:39:12.15" personId="{48458BD6-4CAC-498F-B01C-BB6F89FD41FA}" id="{CDBBDAF0-DC8A-4716-92BA-AC44BC912388}">
+    <text>Divide it by 2e10-3</text>
+  </threadedComment>
   <threadedComment ref="B18" dT="2024-08-07T13:14:12.40" personId="{48458BD6-4CAC-498F-B01C-BB6F89FD41FA}" id="{B6F8C469-337C-40BE-B2DC-A13B6B68197A}">
     <text>Not modelled currently; we specify different off rates depending on whether camkii is P or not.</text>
   </threadedComment>
@@ -1401,49 +1419,49 @@
         <v>0</v>
       </c>
       <c r="B1" s="36" t="s">
-        <v>14</v>
+        <v>12</v>
       </c>
       <c r="C1" s="36" t="s">
-        <v>15</v>
+        <v>13</v>
       </c>
       <c r="D1" s="36" t="s">
         <v>2</v>
       </c>
       <c r="E1" s="36" t="s">
-        <v>15</v>
+        <v>13</v>
       </c>
       <c r="F1" s="36" t="s">
         <v>2</v>
       </c>
       <c r="G1" s="36" t="s">
-        <v>15</v>
+        <v>13</v>
       </c>
       <c r="H1" s="36" t="s">
-        <v>20</v>
+        <v>18</v>
       </c>
       <c r="I1" s="36" t="s">
         <v>2</v>
       </c>
       <c r="J1" s="36" t="s">
-        <v>15</v>
+        <v>13</v>
       </c>
       <c r="K1" s="36" t="s">
         <v>2</v>
       </c>
       <c r="L1" s="36" t="s">
-        <v>15</v>
+        <v>13</v>
       </c>
       <c r="M1" s="36" t="s">
         <v>2</v>
       </c>
       <c r="N1" s="36" t="s">
-        <v>15</v>
+        <v>13</v>
       </c>
       <c r="O1" s="36" t="s">
         <v>2</v>
       </c>
       <c r="P1" s="36" t="s">
-        <v>15</v>
+        <v>13</v>
       </c>
       <c r="Q1" s="36" t="s">
         <v>2</v>
@@ -1451,22 +1469,22 @@
     </row>
     <row r="2" spans="1:101" s="2" customFormat="1" ht="15.75" thickTop="1" x14ac:dyDescent="0.25">
       <c r="A2" s="12" t="s">
-        <v>40</v>
+        <v>38</v>
       </c>
       <c r="B2" s="6" t="s">
-        <v>26</v>
+        <v>24</v>
       </c>
       <c r="C2" s="17">
         <v>1000000</v>
       </c>
       <c r="D2" s="18" t="s">
-        <v>16</v>
+        <v>14</v>
       </c>
       <c r="E2" s="17">
         <v>257000000</v>
       </c>
       <c r="F2" s="18" t="s">
-        <v>51</v>
+        <v>49</v>
       </c>
       <c r="G2" s="29">
         <v>25000000</v>
@@ -1475,31 +1493,31 @@
         <v>260000000</v>
       </c>
       <c r="I2" s="30" t="s">
-        <v>19</v>
+        <v>17</v>
       </c>
       <c r="J2" s="17">
         <v>770000000</v>
       </c>
       <c r="K2" s="18" t="s">
-        <v>18</v>
+        <v>16</v>
       </c>
       <c r="L2" s="24">
         <v>32200000000</v>
       </c>
       <c r="M2" s="25" t="s">
-        <v>21</v>
+        <v>19</v>
       </c>
       <c r="N2" s="33">
         <v>100000000</v>
       </c>
       <c r="O2" s="34" t="s">
-        <v>17</v>
+        <v>15</v>
       </c>
       <c r="P2" s="24">
         <v>100000000</v>
       </c>
       <c r="Q2" s="27" t="s">
-        <v>22</v>
+        <v>20</v>
       </c>
       <c r="R2"/>
       <c r="S2"/>
@@ -1589,19 +1607,19 @@
     <row r="3" spans="1:101" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A3" s="12"/>
       <c r="B3" s="6" t="s">
-        <v>27</v>
+        <v>25</v>
       </c>
       <c r="C3" s="17">
         <v>1000000</v>
       </c>
       <c r="D3" s="18" t="s">
-        <v>16</v>
+        <v>14</v>
       </c>
       <c r="E3" s="17">
         <v>229000</v>
       </c>
       <c r="F3" s="18" t="s">
-        <v>52</v>
+        <v>50</v>
       </c>
       <c r="G3" s="29">
         <v>50000000</v>
@@ -1610,31 +1628,31 @@
         <v>300000000</v>
       </c>
       <c r="I3" s="30" t="s">
-        <v>19</v>
+        <v>17</v>
       </c>
       <c r="J3" s="17">
         <v>32000000000</v>
       </c>
       <c r="K3" s="18" t="s">
-        <v>18</v>
+        <v>16</v>
       </c>
       <c r="L3" s="24">
         <v>32200000000</v>
       </c>
       <c r="M3" s="25" t="s">
-        <v>21</v>
+        <v>19</v>
       </c>
       <c r="N3" s="33">
         <v>150000000</v>
       </c>
       <c r="O3" s="34" t="s">
-        <v>17</v>
+        <v>15</v>
       </c>
       <c r="P3" s="24">
         <v>150000000</v>
       </c>
       <c r="Q3" s="27" t="s">
-        <v>22</v>
+        <v>20</v>
       </c>
       <c r="R3"/>
       <c r="S3"/>
@@ -1724,19 +1742,19 @@
     <row r="4" spans="1:101" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A4" s="12"/>
       <c r="B4" s="6" t="s">
-        <v>24</v>
+        <v>22</v>
       </c>
       <c r="C4" s="17">
         <v>1000000</v>
       </c>
       <c r="D4" s="18" t="s">
-        <v>16</v>
+        <v>14</v>
       </c>
       <c r="E4" s="17">
         <v>21400000</v>
       </c>
       <c r="F4" s="18" t="s">
-        <v>53</v>
+        <v>51</v>
       </c>
       <c r="G4" s="29">
         <v>1200000</v>
@@ -1745,31 +1763,31 @@
         <v>9600000</v>
       </c>
       <c r="I4" s="30" t="s">
-        <v>19</v>
+        <v>17</v>
       </c>
       <c r="J4" s="17">
         <v>84000000</v>
       </c>
       <c r="K4" s="18" t="s">
-        <v>18</v>
+        <v>16</v>
       </c>
       <c r="L4" s="24">
         <v>322000000</v>
       </c>
       <c r="M4" s="25" t="s">
-        <v>21</v>
+        <v>19</v>
       </c>
       <c r="N4" s="33">
         <v>4000000</v>
       </c>
       <c r="O4" s="34" t="s">
-        <v>17</v>
+        <v>15</v>
       </c>
       <c r="P4" s="24">
         <v>4000000</v>
       </c>
       <c r="Q4" s="27" t="s">
-        <v>22</v>
+        <v>20</v>
       </c>
       <c r="R4"/>
       <c r="S4"/>
@@ -1859,19 +1877,19 @@
     <row r="5" spans="1:101" s="2" customFormat="1" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A5" s="12"/>
       <c r="B5" s="6" t="s">
-        <v>25</v>
+        <v>23</v>
       </c>
       <c r="C5" s="17">
         <v>1000000</v>
       </c>
       <c r="D5" s="18" t="s">
-        <v>16</v>
+        <v>14</v>
       </c>
       <c r="E5" s="17">
         <v>110000000</v>
       </c>
       <c r="F5" s="18" t="s">
-        <v>54</v>
+        <v>52</v>
       </c>
       <c r="G5" s="29">
         <v>5000000</v>
@@ -1880,31 +1898,31 @@
         <v>25000000</v>
       </c>
       <c r="I5" s="30" t="s">
-        <v>19</v>
+        <v>17</v>
       </c>
       <c r="J5" s="17">
         <v>250000000</v>
       </c>
       <c r="K5" s="18" t="s">
-        <v>18</v>
+        <v>16</v>
       </c>
       <c r="L5" s="24">
         <v>322000000</v>
       </c>
       <c r="M5" s="25" t="s">
-        <v>21</v>
+        <v>19</v>
       </c>
       <c r="N5" s="33">
         <v>10000000</v>
       </c>
       <c r="O5" s="34" t="s">
-        <v>17</v>
+        <v>15</v>
       </c>
       <c r="P5" s="24">
         <v>10000000</v>
       </c>
       <c r="Q5" s="27" t="s">
-        <v>22</v>
+        <v>20</v>
       </c>
       <c r="R5"/>
       <c r="S5"/>
@@ -1993,50 +2011,50 @@
     </row>
     <row r="6" spans="1:101" s="2" customFormat="1" ht="16.5" thickTop="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A6" s="12" t="s">
-        <v>39</v>
+        <v>37</v>
       </c>
       <c r="B6" s="36" t="s">
         <v>1</v>
       </c>
       <c r="C6" s="36" t="s">
-        <v>23</v>
+        <v>21</v>
       </c>
       <c r="D6" s="36" t="s">
         <v>2</v>
       </c>
       <c r="E6" s="36" t="s">
-        <v>23</v>
+        <v>21</v>
       </c>
       <c r="F6" s="36"/>
       <c r="G6" s="36" t="s">
-        <v>23</v>
+        <v>21</v>
       </c>
       <c r="H6" s="36" t="s">
-        <v>20</v>
+        <v>18</v>
       </c>
       <c r="I6" s="36" t="s">
         <v>2</v>
       </c>
       <c r="J6" s="36" t="s">
-        <v>23</v>
+        <v>21</v>
       </c>
       <c r="K6" s="36" t="s">
         <v>2</v>
       </c>
       <c r="L6" s="36" t="s">
-        <v>32</v>
+        <v>30</v>
       </c>
       <c r="M6" s="36" t="s">
         <v>2</v>
       </c>
       <c r="N6" s="36" t="s">
-        <v>23</v>
+        <v>21</v>
       </c>
       <c r="O6" s="36" t="s">
         <v>2</v>
       </c>
       <c r="P6" s="36" t="s">
-        <v>23</v>
+        <v>21</v>
       </c>
       <c r="Q6" s="36" t="s">
         <v>2</v>
@@ -2129,19 +2147,19 @@
     <row r="7" spans="1:101" s="2" customFormat="1" ht="15.75" thickTop="1" x14ac:dyDescent="0.25">
       <c r="A7" s="12"/>
       <c r="B7" s="6" t="s">
-        <v>28</v>
+        <v>26</v>
       </c>
       <c r="C7" s="19">
         <v>1.9279999999999999</v>
       </c>
       <c r="D7" s="20" t="s">
-        <v>16</v>
+        <v>14</v>
       </c>
       <c r="E7" s="17">
         <v>2040</v>
       </c>
       <c r="F7" s="18" t="s">
-        <v>51</v>
+        <v>49</v>
       </c>
       <c r="G7" s="29">
         <v>1000</v>
@@ -2150,31 +2168,31 @@
         <v>4000</v>
       </c>
       <c r="I7" s="30" t="s">
-        <v>19</v>
+        <v>17</v>
       </c>
       <c r="J7" s="17">
         <v>160000</v>
       </c>
       <c r="K7" s="18" t="s">
-        <v>18</v>
+        <v>16</v>
       </c>
       <c r="L7" s="26">
         <v>9.3800000000000003E-5</v>
       </c>
       <c r="M7" s="25" t="s">
-        <v>21</v>
+        <v>19</v>
       </c>
       <c r="N7" s="33">
         <v>2660</v>
       </c>
       <c r="O7" s="34" t="s">
-        <v>17</v>
+        <v>15</v>
       </c>
       <c r="P7" s="24">
         <v>2660</v>
       </c>
       <c r="Q7" s="27" t="s">
-        <v>22</v>
+        <v>20</v>
       </c>
       <c r="R7"/>
       <c r="S7"/>
@@ -2264,19 +2282,19 @@
     <row r="8" spans="1:101" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A8" s="12"/>
       <c r="B8" s="6" t="s">
-        <v>29</v>
+        <v>27</v>
       </c>
       <c r="C8" s="19">
         <v>1.9370000000000001</v>
       </c>
       <c r="D8" s="20" t="s">
-        <v>16</v>
+        <v>14</v>
       </c>
       <c r="E8" s="17">
         <v>0.39</v>
       </c>
       <c r="F8" s="18" t="s">
-        <v>52</v>
+        <v>50</v>
       </c>
       <c r="G8" s="29">
         <v>500</v>
@@ -2285,31 +2303,31 @@
         <v>1000</v>
       </c>
       <c r="I8" s="30" t="s">
-        <v>19</v>
+        <v>17</v>
       </c>
       <c r="J8" s="17">
         <v>22000</v>
       </c>
       <c r="K8" s="18" t="s">
-        <v>18</v>
+        <v>16</v>
       </c>
       <c r="L8" s="26">
         <v>9.3800000000000003E-5</v>
       </c>
       <c r="M8" s="25" t="s">
-        <v>21</v>
+        <v>19</v>
       </c>
       <c r="N8" s="33">
         <v>990</v>
       </c>
       <c r="O8" s="34" t="s">
-        <v>17</v>
+        <v>15</v>
       </c>
       <c r="P8" s="24">
         <v>990</v>
       </c>
       <c r="Q8" s="27" t="s">
-        <v>22</v>
+        <v>20</v>
       </c>
       <c r="R8"/>
       <c r="S8"/>
@@ -2399,19 +2417,19 @@
     <row r="9" spans="1:101" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A9" s="12"/>
       <c r="B9" s="6" t="s">
-        <v>30</v>
+        <v>28</v>
       </c>
       <c r="C9" s="19">
         <v>7.476</v>
       </c>
       <c r="D9" s="20" t="s">
-        <v>16</v>
+        <v>14</v>
       </c>
       <c r="E9" s="17">
         <v>742</v>
       </c>
       <c r="F9" s="18" t="s">
-        <v>53</v>
+        <v>51</v>
       </c>
       <c r="G9" s="31">
         <v>10</v>
@@ -2420,31 +2438,31 @@
         <v>70</v>
       </c>
       <c r="I9" s="30" t="s">
-        <v>19</v>
+        <v>17</v>
       </c>
       <c r="J9" s="17">
         <v>2600</v>
       </c>
       <c r="K9" s="18" t="s">
-        <v>18</v>
+        <v>16</v>
       </c>
       <c r="L9" s="26">
         <v>9.3800000000000003E-5</v>
       </c>
       <c r="M9" s="25" t="s">
-        <v>21</v>
+        <v>19</v>
       </c>
       <c r="N9" s="35">
         <v>40.24</v>
       </c>
       <c r="O9" s="34" t="s">
-        <v>17</v>
+        <v>15</v>
       </c>
       <c r="P9" s="28">
         <v>40.24</v>
       </c>
       <c r="Q9" s="27" t="s">
-        <v>22</v>
+        <v>20</v>
       </c>
       <c r="R9"/>
       <c r="S9"/>
@@ -2534,19 +2552,19 @@
     <row r="10" spans="1:101" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A10" s="12"/>
       <c r="B10" s="6" t="s">
-        <v>31</v>
+        <v>29</v>
       </c>
       <c r="C10" s="19">
         <v>25.783000000000001</v>
       </c>
       <c r="D10" s="20" t="s">
-        <v>16</v>
+        <v>14</v>
       </c>
       <c r="E10" s="17">
         <v>980</v>
       </c>
       <c r="F10" s="18" t="s">
-        <v>54</v>
+        <v>52</v>
       </c>
       <c r="G10" s="31">
         <v>8.5</v>
@@ -2555,31 +2573,31 @@
         <v>10</v>
       </c>
       <c r="I10" s="30" t="s">
-        <v>19</v>
+        <v>17</v>
       </c>
       <c r="J10" s="19">
         <v>6.5</v>
       </c>
       <c r="K10" s="18" t="s">
-        <v>18</v>
+        <v>16</v>
       </c>
       <c r="L10" s="26">
         <v>9.3800000000000003E-5</v>
       </c>
       <c r="M10" s="25" t="s">
-        <v>21</v>
+        <v>19</v>
       </c>
       <c r="N10" s="35">
         <v>9.3000000000000007</v>
       </c>
       <c r="O10" s="34" t="s">
-        <v>17</v>
+        <v>15</v>
       </c>
       <c r="P10" s="28">
         <v>9.3000000000000007</v>
       </c>
       <c r="Q10" s="27" t="s">
-        <v>22</v>
+        <v>20</v>
       </c>
       <c r="R10"/>
       <c r="S10"/>
@@ -2671,13 +2689,13 @@
         <v>3</v>
       </c>
       <c r="B11" s="7" t="s">
-        <v>4</v>
+        <v>55</v>
       </c>
       <c r="C11" s="1">
         <v>20000</v>
       </c>
       <c r="D11" s="13" t="s">
-        <v>12</v>
+        <v>10</v>
       </c>
       <c r="E11" s="13"/>
       <c r="F11" s="13"/>
@@ -2691,13 +2709,13 @@
     <row r="12" spans="1:101" ht="18" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A12" s="11"/>
       <c r="B12" s="7" t="s">
-        <v>5</v>
+        <v>56</v>
       </c>
       <c r="C12" s="1">
         <v>10000000</v>
       </c>
       <c r="D12" s="13" t="s">
-        <v>13</v>
+        <v>11</v>
       </c>
       <c r="E12" s="13"/>
       <c r="F12" s="13"/>
@@ -2711,49 +2729,49 @@
     <row r="13" spans="1:101" ht="18" customHeight="1" thickTop="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A13" s="11"/>
       <c r="B13" s="36" t="s">
-        <v>14</v>
+        <v>12</v>
       </c>
       <c r="C13" s="36" t="s">
-        <v>15</v>
+        <v>13</v>
       </c>
       <c r="D13" s="36" t="s">
         <v>2</v>
       </c>
       <c r="E13" s="36" t="s">
-        <v>15</v>
+        <v>13</v>
       </c>
       <c r="F13" s="36" t="s">
         <v>2</v>
       </c>
       <c r="G13" s="36" t="s">
-        <v>15</v>
+        <v>13</v>
       </c>
       <c r="H13" s="36" t="s">
-        <v>20</v>
+        <v>18</v>
       </c>
       <c r="I13" s="36" t="s">
         <v>2</v>
       </c>
       <c r="J13" s="36" t="s">
-        <v>15</v>
+        <v>13</v>
       </c>
       <c r="K13" s="36" t="s">
         <v>2</v>
       </c>
       <c r="L13" s="36" t="s">
-        <v>15</v>
+        <v>13</v>
       </c>
       <c r="M13" s="36" t="s">
         <v>2</v>
       </c>
       <c r="N13" s="36" t="s">
-        <v>15</v>
+        <v>13</v>
       </c>
       <c r="O13" s="36" t="s">
         <v>2</v>
       </c>
       <c r="P13" s="36" t="s">
-        <v>15</v>
+        <v>13</v>
       </c>
       <c r="Q13" s="36" t="s">
         <v>2</v>
@@ -2761,22 +2779,22 @@
     </row>
     <row r="14" spans="1:101" s="2" customFormat="1" ht="33.75" customHeight="1" thickTop="1" x14ac:dyDescent="0.25">
       <c r="A14" s="12" t="s">
-        <v>42</v>
+        <v>40</v>
       </c>
       <c r="B14" s="6" t="s">
-        <v>6</v>
+        <v>4</v>
       </c>
       <c r="C14" s="21">
         <v>4200000</v>
       </c>
       <c r="D14" s="18" t="s">
-        <v>16</v>
+        <v>14</v>
       </c>
       <c r="E14" s="45" t="s">
-        <v>35</v>
+        <v>33</v>
       </c>
       <c r="F14" s="45" t="s">
-        <v>35</v>
+        <v>33</v>
       </c>
       <c r="G14" s="29">
         <v>1400000</v>
@@ -2785,31 +2803,31 @@
         <v>60000000</v>
       </c>
       <c r="I14" s="30" t="s">
-        <v>19</v>
+        <v>17</v>
       </c>
       <c r="J14" s="51">
         <v>1600000</v>
       </c>
       <c r="K14" s="30" t="s">
-        <v>56</v>
+        <v>54</v>
       </c>
       <c r="L14" s="10">
         <v>2860000</v>
       </c>
       <c r="M14" s="8" t="s">
-        <v>21</v>
+        <v>19</v>
       </c>
       <c r="N14" s="14" t="s">
-        <v>35</v>
+        <v>33</v>
       </c>
       <c r="O14" s="14" t="s">
-        <v>35</v>
+        <v>33</v>
       </c>
       <c r="P14" s="14" t="s">
-        <v>35</v>
+        <v>33</v>
       </c>
       <c r="Q14" s="14" t="s">
-        <v>35</v>
+        <v>33</v>
       </c>
       <c r="R14"/>
       <c r="S14"/>
@@ -2899,52 +2917,52 @@
     <row r="15" spans="1:101" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A15" s="12"/>
       <c r="B15" s="6" t="s">
-        <v>36</v>
+        <v>34</v>
       </c>
       <c r="C15" s="14" t="s">
-        <v>35</v>
+        <v>33</v>
       </c>
       <c r="D15" s="45" t="s">
-        <v>35</v>
+        <v>33</v>
       </c>
       <c r="E15" s="48">
         <v>150000000</v>
       </c>
       <c r="F15" s="49" t="s">
-        <v>55</v>
+        <v>53</v>
       </c>
       <c r="G15" s="29" t="s">
-        <v>35</v>
+        <v>33</v>
       </c>
       <c r="H15" s="29" t="s">
-        <v>35</v>
+        <v>33</v>
       </c>
       <c r="I15" s="30" t="s">
-        <v>35</v>
+        <v>33</v>
       </c>
       <c r="J15" s="52">
         <v>3400000</v>
       </c>
       <c r="K15" s="3" t="s">
-        <v>35</v>
+        <v>33</v>
       </c>
       <c r="L15" s="10" t="s">
-        <v>35</v>
+        <v>33</v>
       </c>
       <c r="M15" s="8" t="s">
-        <v>35</v>
+        <v>33</v>
       </c>
       <c r="N15" s="33">
         <v>30000000</v>
       </c>
       <c r="O15" s="34" t="s">
-        <v>17</v>
+        <v>15</v>
       </c>
       <c r="P15" s="24">
         <v>30000000</v>
       </c>
       <c r="Q15" s="27" t="s">
-        <v>22</v>
+        <v>20</v>
       </c>
       <c r="R15"/>
       <c r="S15" s="15"/>
@@ -3034,52 +3052,52 @@
     <row r="16" spans="1:101" s="2" customFormat="1" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A16" s="12"/>
       <c r="B16" s="6" t="s">
-        <v>37</v>
+        <v>35</v>
       </c>
       <c r="C16" s="14" t="s">
-        <v>35</v>
+        <v>33</v>
       </c>
       <c r="D16" s="45" t="s">
-        <v>35</v>
+        <v>33</v>
       </c>
       <c r="E16" s="48">
         <v>50000000</v>
       </c>
       <c r="F16" s="49" t="s">
-        <v>55</v>
+        <v>53</v>
       </c>
       <c r="G16" s="29" t="s">
-        <v>35</v>
+        <v>33</v>
       </c>
       <c r="H16" s="29" t="s">
-        <v>35</v>
+        <v>33</v>
       </c>
       <c r="I16" s="30" t="s">
-        <v>35</v>
+        <v>33</v>
       </c>
       <c r="J16" s="3" t="s">
-        <v>35</v>
+        <v>33</v>
       </c>
       <c r="K16" s="3" t="s">
-        <v>35</v>
+        <v>33</v>
       </c>
       <c r="L16" s="10" t="s">
-        <v>35</v>
+        <v>33</v>
       </c>
       <c r="M16" s="8" t="s">
-        <v>35</v>
+        <v>33</v>
       </c>
       <c r="N16" s="33">
         <v>10000000</v>
       </c>
       <c r="O16" s="34" t="s">
-        <v>17</v>
+        <v>15</v>
       </c>
       <c r="P16" s="24">
         <v>50000000</v>
       </c>
       <c r="Q16" s="27" t="s">
-        <v>22</v>
+        <v>20</v>
       </c>
       <c r="R16"/>
       <c r="S16" s="15"/>
@@ -3172,46 +3190,46 @@
         <v>1</v>
       </c>
       <c r="C17" s="36" t="s">
-        <v>23</v>
+        <v>21</v>
       </c>
       <c r="D17" s="36" t="s">
         <v>2</v>
       </c>
       <c r="E17" s="36" t="s">
-        <v>23</v>
+        <v>21</v>
       </c>
       <c r="F17" s="36" t="s">
         <v>2</v>
       </c>
       <c r="G17" s="36" t="s">
-        <v>23</v>
+        <v>21</v>
       </c>
       <c r="H17" s="36" t="s">
-        <v>20</v>
+        <v>18</v>
       </c>
       <c r="I17" s="36" t="s">
         <v>2</v>
       </c>
       <c r="J17" s="36" t="s">
-        <v>23</v>
+        <v>21</v>
       </c>
       <c r="K17" s="36" t="s">
         <v>2</v>
       </c>
       <c r="L17" s="36" t="s">
-        <v>32</v>
+        <v>30</v>
       </c>
       <c r="M17" s="36" t="s">
         <v>2</v>
       </c>
       <c r="N17" s="36" t="s">
-        <v>23</v>
+        <v>21</v>
       </c>
       <c r="O17" s="36" t="s">
         <v>2</v>
       </c>
       <c r="P17" s="36" t="s">
-        <v>23</v>
+        <v>21</v>
       </c>
       <c r="Q17" s="36" t="s">
         <v>2</v>
@@ -3303,22 +3321,22 @@
     </row>
     <row r="18" spans="1:101" ht="30.75" thickTop="1" x14ac:dyDescent="0.25">
       <c r="A18" s="11" t="s">
-        <v>41</v>
+        <v>39</v>
       </c>
       <c r="B18" s="7" t="s">
-        <v>33</v>
+        <v>31</v>
       </c>
       <c r="C18" s="17">
         <v>2.5000000000000001E-4</v>
       </c>
       <c r="D18" s="20" t="s">
-        <v>16</v>
+        <v>14</v>
       </c>
       <c r="E18" s="45" t="s">
-        <v>35</v>
+        <v>33</v>
       </c>
       <c r="F18" s="45" t="s">
-        <v>35</v>
+        <v>33</v>
       </c>
       <c r="G18" s="31">
         <v>1.1000000000000001</v>
@@ -3327,142 +3345,142 @@
         <v>2.2999999999999998</v>
       </c>
       <c r="I18" s="30" t="s">
-        <v>19</v>
+        <v>17</v>
       </c>
       <c r="J18" s="2" t="s">
-        <v>34</v>
+        <v>32</v>
       </c>
       <c r="K18" s="2" t="s">
-        <v>34</v>
+        <v>32</v>
       </c>
       <c r="L18" s="9">
         <v>1.1000000000000001</v>
       </c>
       <c r="M18" s="8" t="s">
-        <v>21</v>
+        <v>19</v>
       </c>
       <c r="N18" s="35" t="s">
-        <v>34</v>
+        <v>32</v>
       </c>
       <c r="O18" s="35" t="s">
-        <v>34</v>
+        <v>32</v>
       </c>
       <c r="P18" s="28" t="s">
-        <v>34</v>
+        <v>32</v>
       </c>
       <c r="Q18" s="27" t="s">
-        <v>34</v>
+        <v>32</v>
       </c>
     </row>
     <row r="19" spans="1:101" x14ac:dyDescent="0.25">
       <c r="A19" s="11"/>
       <c r="B19" s="7" t="s">
-        <v>7</v>
+        <v>5</v>
       </c>
       <c r="C19" s="46" t="s">
-        <v>34</v>
+        <v>32</v>
       </c>
       <c r="D19" s="47" t="s">
-        <v>34</v>
+        <v>32</v>
       </c>
       <c r="E19" s="50">
         <v>0.46</v>
       </c>
       <c r="F19" s="49" t="s">
-        <v>55</v>
+        <v>53</v>
       </c>
       <c r="G19" s="31" t="s">
-        <v>34</v>
+        <v>32</v>
       </c>
       <c r="H19" s="31" t="s">
-        <v>34</v>
+        <v>32</v>
       </c>
       <c r="I19" s="30" t="s">
-        <v>34</v>
+        <v>32</v>
       </c>
       <c r="J19" s="2" t="s">
-        <v>34</v>
+        <v>32</v>
       </c>
       <c r="K19" s="2" t="s">
-        <v>34</v>
+        <v>32</v>
       </c>
       <c r="L19" s="9" t="s">
-        <v>34</v>
+        <v>32</v>
       </c>
       <c r="M19" s="8" t="s">
-        <v>34</v>
+        <v>32</v>
       </c>
       <c r="N19" s="35">
         <v>1.95</v>
       </c>
       <c r="O19" s="34" t="s">
-        <v>17</v>
+        <v>15</v>
       </c>
       <c r="P19" s="28">
         <v>1.95</v>
       </c>
       <c r="Q19" s="27" t="s">
-        <v>22</v>
+        <v>20</v>
       </c>
     </row>
     <row r="20" spans="1:101" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A20" s="11"/>
       <c r="B20" s="7" t="s">
-        <v>8</v>
+        <v>6</v>
       </c>
       <c r="C20" s="46" t="s">
-        <v>34</v>
+        <v>32</v>
       </c>
       <c r="D20" s="47" t="s">
-        <v>34</v>
+        <v>32</v>
       </c>
       <c r="E20" s="48">
         <v>1000</v>
       </c>
       <c r="F20" s="49" t="s">
-        <v>55</v>
+        <v>53</v>
       </c>
       <c r="G20" s="31" t="s">
-        <v>34</v>
+        <v>32</v>
       </c>
       <c r="H20" s="31" t="s">
-        <v>34</v>
+        <v>32</v>
       </c>
       <c r="I20" s="30" t="s">
-        <v>34</v>
+        <v>32</v>
       </c>
       <c r="J20" s="2" t="s">
-        <v>34</v>
+        <v>32</v>
       </c>
       <c r="K20" s="2" t="s">
-        <v>34</v>
+        <v>32</v>
       </c>
       <c r="L20" s="9" t="s">
-        <v>34</v>
+        <v>32</v>
       </c>
       <c r="M20" s="8" t="s">
-        <v>34</v>
+        <v>32</v>
       </c>
       <c r="N20" s="35">
         <v>7.0000000000000007E-2</v>
       </c>
       <c r="O20" s="34" t="s">
-        <v>17</v>
+        <v>15</v>
       </c>
       <c r="P20" s="24">
         <v>9.0000000000000006E-5</v>
       </c>
       <c r="Q20" s="27" t="s">
-        <v>22</v>
+        <v>20</v>
       </c>
     </row>
     <row r="21" spans="1:101" ht="16.5" thickTop="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A21" s="11"/>
       <c r="B21" s="36" t="s">
-        <v>14</v>
+        <v>12</v>
       </c>
       <c r="C21" s="36" t="s">
-        <v>23</v>
+        <v>21</v>
       </c>
       <c r="D21" s="36" t="s">
         <v>2</v>
@@ -3470,34 +3488,34 @@
       <c r="E21" s="36"/>
       <c r="F21" s="36"/>
       <c r="G21" s="36" t="s">
-        <v>23</v>
+        <v>21</v>
       </c>
       <c r="H21" s="36" t="s">
-        <v>20</v>
+        <v>18</v>
       </c>
       <c r="I21" s="36" t="s">
         <v>2</v>
       </c>
       <c r="J21" s="36" t="s">
-        <v>23</v>
+        <v>21</v>
       </c>
       <c r="K21" s="36" t="s">
         <v>2</v>
       </c>
       <c r="L21" s="36" t="s">
-        <v>15</v>
+        <v>13</v>
       </c>
       <c r="M21" s="36" t="s">
         <v>2</v>
       </c>
       <c r="N21" s="36" t="s">
-        <v>23</v>
+        <v>21</v>
       </c>
       <c r="O21" s="36" t="s">
         <v>2</v>
       </c>
       <c r="P21" s="36" t="s">
-        <v>23</v>
+        <v>21</v>
       </c>
       <c r="Q21" s="36" t="s">
         <v>2</v>
@@ -3505,16 +3523,16 @@
     </row>
     <row r="22" spans="1:101" s="2" customFormat="1" ht="15.75" thickTop="1" x14ac:dyDescent="0.25">
       <c r="A22" s="12" t="s">
-        <v>9</v>
+        <v>7</v>
       </c>
       <c r="B22" s="6" t="s">
-        <v>48</v>
+        <v>46</v>
       </c>
       <c r="C22" s="23">
         <v>10</v>
       </c>
       <c r="D22" s="22" t="s">
-        <v>38</v>
+        <v>36</v>
       </c>
       <c r="E22" s="22"/>
       <c r="F22" s="22"/>
@@ -3525,26 +3543,26 @@
         <v>1.25</v>
       </c>
       <c r="I22" s="30" t="s">
-        <v>19</v>
+        <v>17</v>
       </c>
       <c r="J22" s="2" t="s">
-        <v>34</v>
+        <v>32</v>
       </c>
       <c r="K22" s="2" t="s">
-        <v>34</v>
+        <v>32</v>
       </c>
       <c r="L22" s="3"/>
       <c r="N22" s="35">
         <v>0.96</v>
       </c>
       <c r="O22" s="34" t="s">
-        <v>17</v>
+        <v>15</v>
       </c>
       <c r="P22" s="28">
         <v>0.96</v>
       </c>
       <c r="Q22" s="27" t="s">
-        <v>22</v>
+        <v>20</v>
       </c>
       <c r="R22"/>
       <c r="S22"/>
@@ -3601,16 +3619,16 @@
     </row>
     <row r="23" spans="1:101" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A23" s="11" t="s">
-        <v>10</v>
+        <v>8</v>
       </c>
       <c r="B23" s="7" t="s">
-        <v>49</v>
+        <v>47</v>
       </c>
       <c r="C23" s="39">
         <v>0.02</v>
       </c>
       <c r="D23" s="22" t="s">
-        <v>13</v>
+        <v>11</v>
       </c>
       <c r="E23" s="22"/>
       <c r="F23" s="22"/>
@@ -3621,25 +3639,25 @@
         <v>0.05</v>
       </c>
       <c r="I23" s="43" t="s">
+        <v>42</v>
+      </c>
+      <c r="J23" s="40" t="s">
+        <v>43</v>
+      </c>
+      <c r="K23" s="41" t="s">
         <v>44</v>
       </c>
-      <c r="J23" s="40" t="s">
-        <v>45</v>
-      </c>
-      <c r="K23" s="41" t="s">
-        <v>46</v>
-      </c>
       <c r="N23" s="35" t="s">
-        <v>34</v>
+        <v>32</v>
       </c>
       <c r="O23" s="35" t="s">
-        <v>34</v>
+        <v>32</v>
       </c>
       <c r="P23" s="28" t="s">
-        <v>34</v>
+        <v>32</v>
       </c>
       <c r="Q23" s="28" t="s">
-        <v>34</v>
+        <v>32</v>
       </c>
     </row>
     <row r="24" spans="1:101" ht="16.5" thickTop="1" thickBot="1" x14ac:dyDescent="0.3">
@@ -3648,7 +3666,7 @@
         <v>1</v>
       </c>
       <c r="C24" s="36" t="s">
-        <v>23</v>
+        <v>21</v>
       </c>
       <c r="D24" s="36" t="s">
         <v>2</v>
@@ -3656,34 +3674,34 @@
       <c r="E24" s="36"/>
       <c r="F24" s="36"/>
       <c r="G24" s="36" t="s">
-        <v>23</v>
+        <v>21</v>
       </c>
       <c r="H24" s="36" t="s">
-        <v>20</v>
+        <v>18</v>
       </c>
       <c r="I24" s="36" t="s">
         <v>2</v>
       </c>
       <c r="J24" s="36" t="s">
-        <v>23</v>
+        <v>21</v>
       </c>
       <c r="K24" s="36" t="s">
         <v>2</v>
       </c>
       <c r="L24" s="36" t="s">
-        <v>32</v>
+        <v>30</v>
       </c>
       <c r="M24" s="36" t="s">
         <v>2</v>
       </c>
       <c r="N24" s="36" t="s">
-        <v>23</v>
+        <v>21</v>
       </c>
       <c r="O24" s="36" t="s">
         <v>2</v>
       </c>
       <c r="P24" s="36" t="s">
-        <v>23</v>
+        <v>21</v>
       </c>
       <c r="Q24" s="16" t="s">
         <v>2</v>
@@ -3691,16 +3709,16 @@
     </row>
     <row r="25" spans="1:101" s="2" customFormat="1" ht="15.75" thickTop="1" x14ac:dyDescent="0.25">
       <c r="A25" s="12" t="s">
-        <v>11</v>
+        <v>9</v>
       </c>
       <c r="B25" s="6" t="s">
-        <v>50</v>
+        <v>48</v>
       </c>
       <c r="C25" s="37">
         <v>20</v>
       </c>
       <c r="D25" s="22" t="s">
-        <v>38</v>
+        <v>36</v>
       </c>
       <c r="E25" s="22"/>
       <c r="F25" s="22"/>
@@ -3714,7 +3732,7 @@
         <v>0.41</v>
       </c>
       <c r="O25" s="34" t="s">
-        <v>17</v>
+        <v>15</v>
       </c>
       <c r="P25" s="23">
         <v>11.5</v>
@@ -3775,12 +3793,12 @@
     </row>
     <row r="26" spans="1:101" x14ac:dyDescent="0.25">
       <c r="A26" s="4" t="s">
-        <v>43</v>
+        <v>41</v>
       </c>
     </row>
     <row r="27" spans="1:101" x14ac:dyDescent="0.25">
       <c r="A27" s="4" t="s">
-        <v>47</v>
+        <v>45</v>
       </c>
     </row>
   </sheetData>

</xml_diff>